<commit_message>
filename fix, result file with arg , lr fix
</commit_message>
<xml_diff>
--- a/cnn results/cnn result - epsilon.xlsx
+++ b/cnn results/cnn result - epsilon.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\flight delay\stpn paper\STPN-main\cnn results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1454E7FB-1C95-4AAE-B9D5-8A55CB95BD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{959F6043-D07D-4CA6-B581-63111B757F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7584" yWindow="0" windowWidth="12336" windowHeight="11448" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="6" r:id="rId1"/>
-    <sheet name="udata " sheetId="8" r:id="rId2"/>
-    <sheet name="cdata epsilon" sheetId="7" r:id="rId3"/>
+    <sheet name="time remove" sheetId="10" r:id="rId2"/>
+    <sheet name="time seq len" sheetId="9" r:id="rId3"/>
+    <sheet name="udata " sheetId="8" r:id="rId4"/>
+    <sheet name="cdata epsilon" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="104">
   <si>
     <t>classification_precision</t>
   </si>
@@ -289,6 +291,57 @@
   <si>
     <t>threshold</t>
   </si>
+  <si>
+    <t>time remove</t>
+  </si>
+  <si>
+    <t>cnnopacus_cdata_sigma0_43_train_results_table_20260117_023046 normal</t>
+  </si>
+  <si>
+    <t>timee remov</t>
+  </si>
+  <si>
+    <t>Final_Eps</t>
+  </si>
+  <si>
+    <t>Overall_MAE</t>
+  </si>
+  <si>
+    <t>Arr_MAE</t>
+  </si>
+  <si>
+    <t>Dep_MAE</t>
+  </si>
+  <si>
+    <t>Arr_Del_MAE</t>
+  </si>
+  <si>
+    <t>Dep_Del_MAE</t>
+  </si>
+  <si>
+    <t>Arr_NonDel_MAE</t>
+  </si>
+  <si>
+    <t>Dep_NonDel_MAE</t>
+  </si>
+  <si>
+    <t>Class_Acc</t>
+  </si>
+  <si>
+    <t>Class_F1</t>
+  </si>
+  <si>
+    <t>normal cdata</t>
+  </si>
+  <si>
+    <t>cdata no time</t>
+  </si>
+  <si>
+    <t>if time include, delay mae good, non delay bad</t>
+  </si>
+  <si>
+    <t>Seq Len</t>
+  </si>
 </sst>
 </file>
 
@@ -338,7 +391,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -361,11 +414,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -379,6 +441,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8455,7 +8520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CE66C11-497F-4BAD-A297-C140DE8F8B95}">
-  <dimension ref="A1:W18"/>
+  <dimension ref="A1:W26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -9033,7 +9098,7 @@
         <v>4.24443066860026</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>83</v>
       </c>
@@ -9065,7 +9130,7 @@
         <v>4.8723999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>84</v>
       </c>
@@ -9095,6 +9160,176 @@
       </c>
       <c r="J18" s="2">
         <v>3.8397000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="P24" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R24" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T24" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="U24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="V24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="W24" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" s="3">
+        <v>7.3646261980491197</v>
+      </c>
+      <c r="C25" s="2">
+        <v>0.72259408111067802</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.54226424862108402</v>
+      </c>
+      <c r="E25" s="2">
+        <v>8.7051407717552696</v>
+      </c>
+      <c r="F25" s="2">
+        <v>4.3567055869653597</v>
+      </c>
+      <c r="G25" s="2">
+        <v>5.40894905246126</v>
+      </c>
+      <c r="H25" s="2">
+        <v>11.203591800959</v>
+      </c>
+      <c r="I25" s="2">
+        <v>6.0297271615041899</v>
+      </c>
+      <c r="J25" s="2">
+        <v>7.6114010142308297</v>
+      </c>
+      <c r="K25" s="2">
+        <v>5059.42527604103</v>
+      </c>
+      <c r="L25" s="2">
+        <v>1422.63944673538</v>
+      </c>
+      <c r="M25" s="2">
+        <v>1966.33158445358</v>
+      </c>
+      <c r="N25" s="2">
+        <v>7.5</v>
+      </c>
+      <c r="O25" s="2">
+        <v>5474</v>
+      </c>
+      <c r="P25" s="2">
+        <v>140.806605120499</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>8448.3963072299903</v>
+      </c>
+      <c r="R25" s="2">
+        <v>19207</v>
+      </c>
+      <c r="S25" s="2">
+        <v>2727</v>
+      </c>
+      <c r="T25" s="2">
+        <v>0.45118419132707899</v>
+      </c>
+      <c r="U25" s="2">
+        <v>0.68181311317981697</v>
+      </c>
+      <c r="V25" s="2">
+        <v>132461</v>
+      </c>
+      <c r="W25" s="2">
+        <v>414939</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26">
+        <v>7.5</v>
+      </c>
+      <c r="C26">
+        <v>0.7137</v>
+      </c>
+      <c r="D26">
+        <v>0.54390000000000005</v>
+      </c>
+      <c r="E26">
+        <v>4.77029465956387</v>
+      </c>
+      <c r="F26">
+        <v>5.2037000000000004</v>
+      </c>
+      <c r="G26">
+        <v>5.66289482818891</v>
       </c>
     </row>
   </sheetData>
@@ -9105,6 +9340,390 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BABFDE7E-B98D-4DEB-8254-0F537CE2C12A}">
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:12" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>23.976900000000001</v>
+      </c>
+      <c r="B2" s="2">
+        <v>5.6333000000000002</v>
+      </c>
+      <c r="C2" s="2">
+        <v>6.0507</v>
+      </c>
+      <c r="D2" s="2">
+        <v>5.2159000000000004</v>
+      </c>
+      <c r="E2" s="2">
+        <v>8.5611999999999995</v>
+      </c>
+      <c r="F2" s="2">
+        <v>8.5363000000000007</v>
+      </c>
+      <c r="G2" s="2">
+        <v>5.1504000000000003</v>
+      </c>
+      <c r="H2" s="2">
+        <v>4.2793999999999999</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0.71479999999999999</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0.54039999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>1.9676</v>
+      </c>
+      <c r="B3" s="2">
+        <v>5.7225000000000001</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5.9486999999999997</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5.4962999999999997</v>
+      </c>
+      <c r="E3" s="2">
+        <v>8.7637999999999998</v>
+      </c>
+      <c r="F3" s="2">
+        <v>8.2978000000000005</v>
+      </c>
+      <c r="G3" s="2">
+        <v>4.9390999999999998</v>
+      </c>
+      <c r="H3" s="2">
+        <v>4.7061000000000002</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0.70850000000000002</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0.53610000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="1:12" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="J7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1.99</v>
+      </c>
+      <c r="B8">
+        <v>5.8423999999999996</v>
+      </c>
+      <c r="C8">
+        <v>6.1235999999999997</v>
+      </c>
+      <c r="D8">
+        <v>5.5610999999999997</v>
+      </c>
+      <c r="E8">
+        <v>8.5336999999999996</v>
+      </c>
+      <c r="F8">
+        <v>8.2574000000000005</v>
+      </c>
+      <c r="G8">
+        <v>5.2592999999999996</v>
+      </c>
+      <c r="H8">
+        <v>4.8006000000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>24.995999999999999</v>
+      </c>
+      <c r="B9">
+        <v>5.7522000000000002</v>
+      </c>
+      <c r="C9">
+        <v>6.2754000000000003</v>
+      </c>
+      <c r="D9">
+        <v>5.2289000000000003</v>
+      </c>
+      <c r="E9">
+        <v>8.2964000000000002</v>
+      </c>
+      <c r="F9">
+        <v>8.5945</v>
+      </c>
+      <c r="G9">
+        <v>5.5506000000000002</v>
+      </c>
+      <c r="H9">
+        <v>4.2797000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A79FCFF4-555F-46BC-B8A3-8309F0EF1E3D}">
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G1" t="s">
+        <v>95</v>
+      </c>
+      <c r="H1" t="s">
+        <v>96</v>
+      </c>
+      <c r="I1" t="s">
+        <v>97</v>
+      </c>
+      <c r="J1" t="s">
+        <v>98</v>
+      </c>
+      <c r="K1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>18</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>5.5339999999999998</v>
+      </c>
+      <c r="D2">
+        <v>5.702</v>
+      </c>
+      <c r="E2">
+        <v>5.367</v>
+      </c>
+      <c r="F2">
+        <v>7.7709999999999999</v>
+      </c>
+      <c r="G2">
+        <v>7.8609999999999998</v>
+      </c>
+      <c r="H2">
+        <v>4.9589999999999996</v>
+      </c>
+      <c r="I2">
+        <v>4.6619999999999999</v>
+      </c>
+      <c r="J2">
+        <v>0.73699999999999999</v>
+      </c>
+      <c r="K2">
+        <v>0.59199999999999997</v>
+      </c>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>6.6689999999999996</v>
+      </c>
+      <c r="D3">
+        <v>7.0490000000000004</v>
+      </c>
+      <c r="E3">
+        <v>6.2889999999999997</v>
+      </c>
+      <c r="F3">
+        <v>7.7350000000000003</v>
+      </c>
+      <c r="G3">
+        <v>7.8159999999999998</v>
+      </c>
+      <c r="H3">
+        <v>6.8019999999999996</v>
+      </c>
+      <c r="I3">
+        <v>5.8579999999999997</v>
+      </c>
+      <c r="J3">
+        <v>0.69499999999999995</v>
+      </c>
+      <c r="K3">
+        <v>0.55400000000000005</v>
+      </c>
+      <c r="L3" s="2"/>
+    </row>
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>24</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>5.5270000000000001</v>
+      </c>
+      <c r="D4">
+        <v>5.7480000000000002</v>
+      </c>
+      <c r="E4">
+        <v>5.306</v>
+      </c>
+      <c r="F4">
+        <v>7.6840000000000002</v>
+      </c>
+      <c r="G4">
+        <v>7.6619999999999999</v>
+      </c>
+      <c r="H4">
+        <v>5.0529999999999999</v>
+      </c>
+      <c r="I4">
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="J4">
+        <v>0.73699999999999999</v>
+      </c>
+      <c r="K4">
+        <v>0.60199999999999998</v>
+      </c>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>6.0620000000000003</v>
+      </c>
+      <c r="D5">
+        <v>6.1929999999999996</v>
+      </c>
+      <c r="E5">
+        <v>5.93</v>
+      </c>
+      <c r="F5">
+        <v>7.96</v>
+      </c>
+      <c r="G5">
+        <v>7.7510000000000003</v>
+      </c>
+      <c r="H5">
+        <v>5.5590000000000002</v>
+      </c>
+      <c r="I5">
+        <v>5.4160000000000004</v>
+      </c>
+      <c r="J5">
+        <v>0.70799999999999996</v>
+      </c>
+      <c r="K5">
+        <v>0.57199999999999995</v>
+      </c>
+      <c r="L5" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3AEABCC-FE12-4367-8399-1B2C82131DA2}">
   <dimension ref="A1:P49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -9670,7 +10289,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28251864-1456-4BBD-958C-1261E9ACD490}">
   <dimension ref="A1:P5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>